<commit_message>
Pre-evaluación de artículos de acceso abierto de Joaquín
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -295,6 +295,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
+    <author>Claude (pre-evaluación 10-10-2026)</author>
   </authors>
   <commentList>
     <comment ref="N4" authorId="0" shapeId="0">
@@ -357,6 +358,11 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
+    <comment ref="L29" authorId="1" shapeId="0">
+      <text>
+        <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): datos reales de 565 000 transferencias de una caja rural de España, RF supera a redes neuronales y Naive Bayes. Pero es FRAUDE, no lavado ni operaciones inusuales, y reporta 'accuracy 100 %' para legítimas (señal de métrica mal elegida). Ronda 4: dudoso, probablemente Sale. Relevancia baja-media.</t>
+      </text>
+    </comment>
     <comment ref="M29" authorId="0" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
@@ -372,9 +378,10 @@
         <t>Implicancias legales</t>
       </text>
     </comment>
-    <comment ref="M37" authorId="0" shapeId="0">
+    <comment ref="M37" authorId="1" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.
+Corrección: NO es de acceso abierto (licencia solo de minería de texto). Pedirlo por biblioteca UPC.</t>
       </text>
     </comment>
     <comment ref="M39" authorId="0" shapeId="0">
@@ -407,6 +414,11 @@
         <t>Es un survey (CE3)</t>
       </text>
     </comment>
+    <comment ref="L52" authorId="1" shapeId="0">
+      <text>
+        <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.</t>
+      </text>
+    </comment>
     <comment ref="M52" authorId="0" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
@@ -420,6 +432,11 @@
     <comment ref="K77" authorId="0" shapeId="0">
       <text>
         <t>Es un review (CE3)</t>
+      </text>
+    </comment>
+    <comment ref="L81" authorId="1" shapeId="0">
+      <text>
+        <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).</t>
       </text>
     </comment>
     <comment ref="M81" authorId="0" shapeId="0">

</xml_diff>

<commit_message>
Lectura completa de 4 artículos de acceso abierto de Joaquín
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -296,6 +296,7 @@
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
+    <author>Claude (lectura completa 10-10-2026)</author>
   </authors>
   <commentList>
     <comment ref="N4" authorId="0" shapeId="0">
@@ -368,6 +369,11 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
+    <comment ref="N29" authorId="2" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: Sale (ronda 4). Fraude en transferencias (estafas) en una caja rural de España, 565 000 transferencias de 6 semanas, solo 333 fraudes (95 en test). RF: 0 falsos positivos y 91/95 fraudes. No es lavado ni operaciones inusuales; la guía lo excluye. Además no describe variables ni partición temporal, y 0 FP con 95 positivos es poco creíble.</t>
+      </text>
+    </comment>
     <comment ref="L31" authorId="0" shapeId="0">
       <text>
         <t>PDF leído. Banco real de Japón, 2019-2020, RF supervisado, FPR 0,000 / FNR 0,005. Pero detecta transferencias NO AUTORIZADAS (robo de cuentas por phishing), no lavado ni operaciones inusuales del cliente. Ronda 4: probablemente Sale; decidir con el equipo.</t>
@@ -414,9 +420,10 @@
         <t>Es un survey (CE3)</t>
       </text>
     </comment>
-    <comment ref="L52" authorId="1" shapeId="0">
+    <comment ref="L52" authorId="2" shapeId="0">
       <text>
-        <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.</t>
+        <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.
+LECTURA COMPLETA: cumple en lo formal (aporte + experimentos), pero relevancia BAJA-MEDIA. Dinamarca. Solo datos SINTÉTICOS (IBM-AML) y modelos de grafos (FraudGT, GatedGCN) entre muchos bancos. Hallazgo útil para P5: cuando cada entidad ve solo sus datos, el F1 cae de 0,32/0,71 a 0,12/0,56 y los modelos más simples rinden mejor (0,49/0,85). Perumoney es una sola entidad sin grafo entre cuentas. Recomendación: dejarlo de RESERVA; solo entra si faltan artículos y el cuartil es Q1/Q2.</t>
       </text>
     </comment>
     <comment ref="M52" authorId="0" shapeId="0">
@@ -434,9 +441,10 @@
         <t>Es un review (CE3)</t>
       </text>
     </comment>
-    <comment ref="L81" authorId="1" shapeId="0">
+    <comment ref="L81" authorId="2" shapeId="0">
       <text>
-        <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).</t>
+        <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).
+LECTURA COMPLETA (versión aceptada del autor): cumple en lo formal, relevancia BAJA. Malasia/China. Método genérico para construir grafos dinámicos para GNN; prueba con un dataset AML privado (30 M transacciones, origen no declarado), un dataset de crédito alemán y Airbnb. No es cripto (CE4 no aplica). Requiere grafo de transacciones entre cuentas que Perumoney no tiene. Recomendación: Sale en ronda 4.</t>
       </text>
     </comment>
     <comment ref="M81" authorId="0" shapeId="0">
@@ -2740,7 +2748,11 @@
         </is>
       </c>
       <c r="M29" s="11" t="n"/>
-      <c r="N29" s="11" t="n"/>
+      <c r="N29" s="11" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
       <c r="O29" s="11" t="n"/>
       <c r="P29" s="8">
         <f>IF(J29="","",IF(K29="Sale","Descartado",IF(L29="Sale","Descartado",IF(OR(M29="Q3",M29="Q4",M29="No aparece"),"Descartado",IF(N29="Sale","Descartado",IF(O29="Sigue","APROBADO","En proceso"))))))</f>

</xml_diff>

<commit_message>
Lectura de Luo (2024) y Alexandre y Balsa (2023)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -295,8 +295,8 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
+    <author>Claude (lectura completa 10-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
-    <author>Claude (lectura completa 10-10-2026)</author>
   </authors>
   <commentList>
     <comment ref="N4" authorId="0" shapeId="0">
@@ -339,6 +339,11 @@
         <t>PDF leído. MUY RELEVANTE: banco real de Pakistán, 1,77 M transacciones, 9 925 cuentas; NO supervisado (k-means y jerárquico + centralidad de grafos), las etiquetas solo se usan para evaluar: justo el caso de P5. Jerárquico: precisión 0,87, recall 0,83, AUC 0,91. Debilidades: solo 75 cuentas sospechosas, no compara contra reglas. Falta cuartil (IEEE Access) para pasar a rondas 4-5: en mi lectura pasaría ambas.</t>
       </text>
     </comment>
+    <comment ref="L21" authorId="1" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: CUMPLE y es MUY RELEVANTE (falta cuartil; ESWA). Alexandre y Balsa (Univ. de Lisboa, Portugal), banco de Brasil. Sistema multiagente: perfiles de comportamiento transaccional de 2,4 M clientes (30,5 M transacciones de 1 año), k-means en 5 perfiles de riesgo + reglas J48 + reglas legales y de analistas + Índice de Sospecha para PRIORIZAR. Validación con analistas reales: 6 meses (17,1 M transacciones, 3,2 M clientes); de 189 clientes revisados, 89 confirmados sospechosos (47 %), incluidos casos que los sistemas vigentes no detectaban. No necesita etiquetas: análogo directo al IE10 del proyecto. Responde P1, P2, P3, P5. Ojo CE2: es de 2023 (límite de 3 años). Si el cuartil es Q1/Q2, pasa rondas 4 y 5.</t>
+      </text>
+    </comment>
     <comment ref="M21" authorId="0" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
@@ -359,7 +364,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="L29" authorId="1" shapeId="0">
+    <comment ref="L29" authorId="2" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): datos reales de 565 000 transferencias de una caja rural de España, RF supera a redes neuronales y Naive Bayes. Pero es FRAUDE, no lavado ni operaciones inusuales, y reporta 'accuracy 100 %' para legítimas (señal de métrica mal elegida). Ronda 4: dudoso, probablemente Sale. Relevancia baja-media.</t>
       </text>
@@ -369,7 +374,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="N29" authorId="2" shapeId="0">
+    <comment ref="N29" authorId="1" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: Sale (ronda 4). Fraude en transferencias (estafas) en una caja rural de España, 565 000 transferencias de 6 semanas, solo 333 fraudes (95 en test). RF: 0 falsos positivos y 91/95 fraudes. No es lavado ni operaciones inusuales; la guía lo excluye. Además no describe variables ni partición temporal, y 0 FP con 95 positivos es poco creíble.</t>
       </text>
@@ -384,7 +389,7 @@
         <t>Implicancias legales</t>
       </text>
     </comment>
-    <comment ref="M37" authorId="1" shapeId="0">
+    <comment ref="M37" authorId="2" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.
 Corrección: NO es de acceso abierto (licencia solo de minería de texto). Pedirlo por biblioteca UPC.</t>
@@ -420,7 +425,7 @@
         <t>Es un survey (CE3)</t>
       </text>
     </comment>
-    <comment ref="L52" authorId="2" shapeId="0">
+    <comment ref="L52" authorId="1" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.
 LECTURA COMPLETA: cumple en lo formal (aporte + experimentos), pero relevancia BAJA-MEDIA. Dinamarca. Solo datos SINTÉTICOS (IBM-AML) y modelos de grafos (FraudGT, GatedGCN) entre muchos bancos. Hallazgo útil para P5: cuando cada entidad ve solo sus datos, el F1 cae de 0,32/0,71 a 0,12/0,56 y los modelos más simples rinden mejor (0,49/0,85). Perumoney es una sola entidad sin grafo entre cuentas. Recomendación: dejarlo de RESERVA; solo entra si faltan artículos y el cuartil es Q1/Q2.</t>
@@ -441,7 +446,7 @@
         <t>Es un review (CE3)</t>
       </text>
     </comment>
-    <comment ref="L81" authorId="2" shapeId="0">
+    <comment ref="L81" authorId="1" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).
 LECTURA COMPLETA (versión aceptada del autor): cumple en lo formal, relevancia BAJA. Malasia/China. Método genérico para construir grafos dinámicos para GNN; prueba con un dataset AML privado (30 M transacciones, origen no declarado), un dataset de crédito alemán y Airbnb. No es cripto (CE4 no aplica). Requiere grafo de transacciones entre cuentas que Perumoney no tiene. Recomendación: Sale en ronda 4.</t>

</xml_diff>

<commit_message>
Cuartil Q1 de Expert Systems with Applications (Alexandre y Balsa aprobado)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -296,6 +296,7 @@
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
     <author>Claude (lectura completa 10-10-2026)</author>
+    <author>Claude (10-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
   </authors>
   <commentList>
@@ -344,9 +345,9 @@
         <t>LECTURA COMPLETA: CUMPLE y es MUY RELEVANTE (falta cuartil; ESWA). Alexandre y Balsa (Univ. de Lisboa, Portugal), banco de Brasil. Sistema multiagente: perfiles de comportamiento transaccional de 2,4 M clientes (30,5 M transacciones de 1 año), k-means en 5 perfiles de riesgo + reglas J48 + reglas legales y de analistas + Índice de Sospecha para PRIORIZAR. Validación con analistas reales: 6 meses (17,1 M transacciones, 3,2 M clientes); de 189 clientes revisados, 89 confirmados sospechosos (47 %), incluidos casos que los sistemas vigentes no detectaban. No necesita etiquetas: análogo directo al IE10 del proyecto. Responde P1, P2, P3, P5. Ojo CE2: es de 2023 (límite de 3 años). Si el cuartil es Q1/Q2, pasa rondas 4 y 5.</t>
       </text>
     </comment>
-    <comment ref="M21" authorId="0" shapeId="0">
+    <comment ref="M21" authorId="2" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Scimago: Expert Systems with Applications, Q1 en 2023 (Artificial Intelligence, Computer Science Applications, Engineering misc.). Captura: Capturas_Scimago/Expert_Systems_with_Applications.png</t>
       </text>
     </comment>
     <comment ref="K23" authorId="0" shapeId="0">
@@ -364,7 +365,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="L29" authorId="2" shapeId="0">
+    <comment ref="L29" authorId="3" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): datos reales de 565 000 transferencias de una caja rural de España, RF supera a redes neuronales y Naive Bayes. Pero es FRAUDE, no lavado ni operaciones inusuales, y reporta 'accuracy 100 %' para legítimas (señal de métrica mal elegida). Ronda 4: dudoso, probablemente Sale. Relevancia baja-media.</t>
       </text>
@@ -389,15 +390,15 @@
         <t>Implicancias legales</t>
       </text>
     </comment>
-    <comment ref="M37" authorId="2" shapeId="0">
+    <comment ref="M37" authorId="3" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.
 Corrección: NO es de acceso abierto (licencia solo de minería de texto). Pedirlo por biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M39" authorId="0" shapeId="0">
+    <comment ref="M39" authorId="2" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Scimago: Expert Systems with Applications, Q1 en 2025. Falta leer el PDF (rondas 4 y 5).</t>
       </text>
     </comment>
     <comment ref="M41" authorId="0" shapeId="0">
@@ -2196,9 +2197,21 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M21" s="11" t="n"/>
-      <c r="N21" s="11" t="n"/>
-      <c r="O21" s="11" t="n"/>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="N21" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P21" s="8">
         <f>IF(J21="","",IF(K21="Sale","Descartado",IF(L21="Sale","Descartado",IF(OR(M21="Q3",M21="Q4",M21="No aparece"),"Descartado",IF(N21="Sale","Descartado",IF(O21="Sigue","APROBADO","En proceso"))))))</f>
         <v/>
@@ -3444,7 +3457,11 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M39" s="11" t="n"/>
+      <c r="M39" s="11" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="N39" s="11" t="n"/>
       <c r="O39" s="11" t="n"/>
       <c r="P39" s="8">

</xml_diff>

<commit_message>
Cuartiles Scimago de 5 revistas de los preseleccionados de Joaquín
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -406,9 +406,9 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M43" authorId="0" shapeId="0">
+    <comment ref="M43" authorId="2" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Journal of Money Laundering Control 2023: Q2 en Economics, Econometrics and Finance (misc.). Falta leer el PDF.</t>
       </text>
     </comment>
     <comment ref="K45" authorId="0" shapeId="0">
@@ -3741,7 +3741,11 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M43" s="11" t="n"/>
+      <c r="M43" s="11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="N43" s="11" t="n"/>
       <c r="O43" s="11" t="n"/>
       <c r="P43" s="8">

</xml_diff>

<commit_message>
Cuartil Q1 de IEEE Access (Irshad aprobado)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -295,8 +295,8 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
+    <author>Claude (10-10-2026)</author>
     <author>Claude (lectura completa 10-10-2026)</author>
-    <author>Claude (10-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
   </authors>
   <commentList>
@@ -340,12 +340,17 @@
         <t>PDF leído. MUY RELEVANTE: banco real de Pakistán, 1,77 M transacciones, 9 925 cuentas; NO supervisado (k-means y jerárquico + centralidad de grafos), las etiquetas solo se usan para evaluar: justo el caso de P5. Jerárquico: precisión 0,87, recall 0,83, AUC 0,91. Debilidades: solo 75 cuentas sospechosas, no compara contra reglas. Falta cuartil (IEEE Access) para pasar a rondas 4-5: en mi lectura pasaría ambas.</t>
       </text>
     </comment>
-    <comment ref="L21" authorId="1" shapeId="0">
+    <comment ref="M19" authorId="1" shapeId="0">
+      <text>
+        <t>IEEE Access 2024: Q1 (Computer Science misc.).</t>
+      </text>
+    </comment>
+    <comment ref="L21" authorId="2" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: CUMPLE y es MUY RELEVANTE (falta cuartil; ESWA). Alexandre y Balsa (Univ. de Lisboa, Portugal), banco de Brasil. Sistema multiagente: perfiles de comportamiento transaccional de 2,4 M clientes (30,5 M transacciones de 1 año), k-means en 5 perfiles de riesgo + reglas J48 + reglas legales y de analistas + Índice de Sospecha para PRIORIZAR. Validación con analistas reales: 6 meses (17,1 M transacciones, 3,2 M clientes); de 189 clientes revisados, 89 confirmados sospechosos (47 %), incluidos casos que los sistemas vigentes no detectaban. No necesita etiquetas: análogo directo al IE10 del proyecto. Responde P1, P2, P3, P5. Ojo CE2: es de 2023 (límite de 3 años). Si el cuartil es Q1/Q2, pasa rondas 4 y 5.</t>
       </text>
     </comment>
-    <comment ref="M21" authorId="2" shapeId="0">
+    <comment ref="M21" authorId="1" shapeId="0">
       <text>
         <t>Scimago: Expert Systems with Applications, Q1 en 2023 (Artificial Intelligence, Computer Science Applications, Engineering misc.). Captura: Capturas_Scimago/Expert_Systems_with_Applications.png</t>
       </text>
@@ -375,7 +380,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="N29" authorId="1" shapeId="0">
+    <comment ref="N29" authorId="2" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: Sale (ronda 4). Fraude en transferencias (estafas) en una caja rural de España, 565 000 transferencias de 6 semanas, solo 333 fraudes (95 en test). RF: 0 falsos positivos y 91/95 fraudes. No es lavado ni operaciones inusuales; la guía lo excluye. Además no describe variables ni partición temporal, y 0 FP con 95 positivos es poco creíble.</t>
       </text>
@@ -396,7 +401,7 @@
 Corrección: NO es de acceso abierto (licencia solo de minería de texto). Pedirlo por biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M39" authorId="2" shapeId="0">
+    <comment ref="M39" authorId="1" shapeId="0">
       <text>
         <t>Scimago: Expert Systems with Applications, Q1 en 2025. Falta leer el PDF (rondas 4 y 5).</t>
       </text>
@@ -406,7 +411,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M43" authorId="2" shapeId="0">
+    <comment ref="M43" authorId="1" shapeId="0">
       <text>
         <t>Journal of Money Laundering Control 2023: Q2 en Economics, Econometrics and Finance (misc.). Falta leer el PDF.</t>
       </text>
@@ -426,7 +431,7 @@
         <t>Es un survey (CE3)</t>
       </text>
     </comment>
-    <comment ref="L52" authorId="1" shapeId="0">
+    <comment ref="L52" authorId="2" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.
 LECTURA COMPLETA: cumple en lo formal (aporte + experimentos), pero relevancia BAJA-MEDIA. Dinamarca. Solo datos SINTÉTICOS (IBM-AML) y modelos de grafos (FraudGT, GatedGCN) entre muchos bancos. Hallazgo útil para P5: cuando cada entidad ve solo sus datos, el F1 cae de 0,32/0,71 a 0,12/0,56 y los modelos más simples rinden mejor (0,49/0,85). Perumoney es una sola entidad sin grafo entre cuentas. Recomendación: dejarlo de RESERVA; solo entra si faltan artículos y el cuartil es Q1/Q2.</t>
@@ -442,12 +447,17 @@
         <t>PDF leído. FinCEN Files (SAR filtradas, 1999-2017), Reino Unido. Compara supervisados (RF/XGBoost AUC ~0,97) vs Isolation Forest/One-Class SVM (&lt;0,75): útil para P4. Debilidades: la etiqueta la construyen ellos con su propio score de riesgo (parcialmente circular), test de solo 41 casos, transacciones banco-a-banco. Falta cuartil (IEEE Access). Ronda 4: dudoso.</t>
       </text>
     </comment>
+    <comment ref="M55" authorId="1" shapeId="0">
+      <text>
+        <t>IEEE Access 2026: aún no publicado; 2025 = Q1. Artículo de reserva (dudoso en ronda 4).</t>
+      </text>
+    </comment>
     <comment ref="K77" authorId="0" shapeId="0">
       <text>
         <t>Es un review (CE3)</t>
       </text>
     </comment>
-    <comment ref="L81" authorId="1" shapeId="0">
+    <comment ref="L81" authorId="2" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).
 LECTURA COMPLETA (versión aceptada del autor): cumple en lo formal, relevancia BAJA. Malasia/China. Método genérico para construir grafos dinámicos para GNN; prueba con un dataset AML privado (30 M transacciones, origen no declarado), un dataset de crédito alemán y Airbnb. No es cripto (CE4 no aplica). Requiere grafo de transacciones entre cuentas que Perumoney no tiene. Recomendación: Sale en ronda 4.</t>
@@ -2057,9 +2067,21 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M19" s="11" t="n"/>
-      <c r="N19" s="11" t="n"/>
-      <c r="O19" s="11" t="n"/>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P19" s="8">
         <f>IF(J19="","",IF(K19="Sale","Descartado",IF(L19="Sale","Descartado",IF(OR(M19="Q3",M19="Q4",M19="No aparece"),"Descartado",IF(N19="Sale","Descartado",IF(O19="Sigue","APROBADO","En proceso"))))))</f>
         <v/>
@@ -4565,7 +4587,11 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M55" s="11" t="n"/>
+      <c r="M55" s="11" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="N55" s="11" t="n"/>
       <c r="O55" s="11" t="n"/>
       <c r="P55" s="8">

</xml_diff>

<commit_message>
Shih et al. (2025) aprobado y registrado en la Matriz
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -406,6 +406,11 @@
         <t>Scimago: Expert Systems with Applications, Q1 en 2025. Falta leer el PDF (rondas 4 y 5).</t>
       </text>
     </comment>
+    <comment ref="N39" authorId="1" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: CUMPLE (Q1). Pese a decir 'fraud', predice eventos SAR (reporte de operación sospechosa de lavado) a partir de alertas SAM de un banco real de Taiwán, con escenarios definidos según la tipología oficial de LA/FT del regulador. Convierte transacciones irregulares de los 15 días hábiles previos en series regulares, autoencoder con self-attention + GNN de relaciones entre clientes + generación de casos (CVAE/WGAN) para el desbalance. Supervisado (etiqueta = decisión del área legal). Compara con XGBoost y redes profundas: AUPRC 27 % vs 0,66-22,15 % (SAR desde alertas) y 22,9 % vs 2,5-22 % (SAR fuera de alertas). Limitación: un solo banco; requiere relaciones entre clientes. Útil para P2 (variables de ventana temporal), P3, P4 y P5 (AUPRC con datos reales y desbalance).</t>
+      </text>
+    </comment>
     <comment ref="M41" authorId="0" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
@@ -3484,8 +3489,16 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="N39" s="11" t="n"/>
-      <c r="O39" s="11" t="n"/>
+      <c r="N39" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
+      <c r="O39" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P39" s="8">
         <f>IF(J39="","",IF(K39="Sale","Descartado",IF(L39="Sale","Descartado",IF(OR(M39="Q3",M39="Q4",M39="No aparece"),"Descartado",IF(N39="Sale","Descartado",IF(O39="Sigue","APROBADO","En proceso"))))))</f>
         <v/>

</xml_diff>

<commit_message>
Lectura de 4 artículos: PageRank aprobado; FSI y SMoTeF registrados; fila 43 en reserva
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -298,6 +298,7 @@
     <author>Claude (10-10-2026)</author>
     <author>Claude (lectura completa 10-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
+    <author>Claude (11-10-2026)</author>
   </authors>
   <commentList>
     <comment ref="N4" authorId="0" shapeId="0">
@@ -419,6 +420,11 @@
     <comment ref="M43" authorId="1" shapeId="0">
       <text>
         <t>Journal of Money Laundering Control 2023: Q2 en Economics, Econometrics and Finance (misc.). Falta leer el PDF.</t>
+      </text>
+    </comment>
+    <comment ref="N43" authorId="4" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: cumple en lo formal pero DÉBIL -&gt; RESERVA. JMLC 2023 (Q2). Capitol Technology Univ., EE. UU. Árbol de decisión y otros clasificadores para predecir si una transacción sobre el umbral debe reportarse (SAR). Datos SINTÉTICOS (transacciones públicas 'modificadas' para imitar banca minorista de EE. UU.), un solo escenario AML, balanceo con ROSE. Aporte: identifica atributos relevantes para el SAR (P2). Es de 2023 (límite CE2).</t>
       </text>
     </comment>
     <comment ref="K45" authorId="0" shapeId="0">
@@ -3781,7 +3787,11 @@
           <t>Q2</t>
         </is>
       </c>
-      <c r="N43" s="11" t="n"/>
+      <c r="N43" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="O43" s="11" t="n"/>
       <c r="P43" s="8">
         <f>IF(J43="","",IF(K43="Sale","Descartado",IF(L43="Sale","Descartado",IF(OR(M43="Q3",M43="Q4",M43="No aparece"),"Descartado",IF(N43="Sale","Descartado",IF(O43="Sigue","APROBADO","En proceso"))))))</f>

</xml_diff>

<commit_message>
Matriz solo con artículos de Candidatos: entran Ejime y Hayble-Gomes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -3792,7 +3792,11 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="O43" s="11" t="n"/>
+      <c r="O43" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P43" s="8">
         <f>IF(J43="","",IF(K43="Sale","Descartado",IF(L43="Sale","Descartado",IF(OR(M43="Q3",M43="Q4",M43="No aparece"),"Descartado",IF(N43="Sale","Descartado",IF(O43="Sigue","APROBADO","En proceso"))))))</f>
         <v/>
@@ -4615,8 +4619,16 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="N55" s="11" t="n"/>
-      <c r="O55" s="11" t="n"/>
+      <c r="N55" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
+      <c r="O55" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P55" s="8">
         <f>IF(J55="","",IF(K55="Sale","Descartado",IF(L55="Sale","Descartado",IF(OR(M55="Q3",M55="Q4",M55="No aparece"),"Descartado",IF(N55="Sale","Descartado",IF(O55="Sigue","APROBADO","En proceso"))))))</f>
         <v/>

</xml_diff>

<commit_message>
Lectura de las filas 8, 27 y 41 de Candidatos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -295,6 +295,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
+    <author>Claude (12-10-2026)</author>
     <author>Claude (10-10-2026)</author>
     <author>Claude (lectura completa 10-10-2026)</author>
     <author>Claude (pre-evaluación 10-10-2026)</author>
@@ -321,6 +322,11 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
+    <comment ref="N8" authorId="1" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: SALE. Astrova (2023), Tallinn Univ. of Technology, Estonia. Artículo descriptivo/divulgativo: explica retos de reglas y ML y describe el algoritmo Anti-TrustRank con un ejemplo ilustrativo; NO hay datos ni experimentos ni métricas. Incumple CI4 (sin validación) y CI1 en sentido estricto.</t>
+      </text>
+    </comment>
     <comment ref="L10" authorId="0" shapeId="0">
       <text>
         <t>Predice sanciones a PAÍSES (Basel AML Index), no operaciones de clientes</t>
@@ -341,17 +347,17 @@
         <t>PDF leído. MUY RELEVANTE: banco real de Pakistán, 1,77 M transacciones, 9 925 cuentas; NO supervisado (k-means y jerárquico + centralidad de grafos), las etiquetas solo se usan para evaluar: justo el caso de P5. Jerárquico: precisión 0,87, recall 0,83, AUC 0,91. Debilidades: solo 75 cuentas sospechosas, no compara contra reglas. Falta cuartil (IEEE Access) para pasar a rondas 4-5: en mi lectura pasaría ambas.</t>
       </text>
     </comment>
-    <comment ref="M19" authorId="1" shapeId="0">
+    <comment ref="M19" authorId="2" shapeId="0">
       <text>
         <t>IEEE Access 2024: Q1 (Computer Science misc.).</t>
       </text>
     </comment>
-    <comment ref="L21" authorId="2" shapeId="0">
+    <comment ref="L21" authorId="3" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: CUMPLE y es MUY RELEVANTE (falta cuartil; ESWA). Alexandre y Balsa (Univ. de Lisboa, Portugal), banco de Brasil. Sistema multiagente: perfiles de comportamiento transaccional de 2,4 M clientes (30,5 M transacciones de 1 año), k-means en 5 perfiles de riesgo + reglas J48 + reglas legales y de analistas + Índice de Sospecha para PRIORIZAR. Validación con analistas reales: 6 meses (17,1 M transacciones, 3,2 M clientes); de 189 clientes revisados, 89 confirmados sospechosos (47 %), incluidos casos que los sistemas vigentes no detectaban. No necesita etiquetas: análogo directo al IE10 del proyecto. Responde P1, P2, P3, P5. Ojo CE2: es de 2023 (límite de 3 años). Si el cuartil es Q1/Q2, pasa rondas 4 y 5.</t>
       </text>
     </comment>
-    <comment ref="M21" authorId="1" shapeId="0">
+    <comment ref="M21" authorId="2" shapeId="0">
       <text>
         <t>Scimago: Expert Systems with Applications, Q1 en 2023 (Artificial Intelligence, Computer Science Applications, Engineering misc.). Captura: Capturas_Scimago/Expert_Systems_with_Applications.png</t>
       </text>
@@ -371,7 +377,12 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="L29" authorId="3" shapeId="0">
+    <comment ref="N27" authorId="1" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: cumple en lo formal pero DÉBIL. Lokanan (2024; en línea 2022), Royal Roads Univ., Canadá. NB, RF, regresión logística, CatBoost y red neuronal sobre datos SIMULADOS de bancos de Medio Oriente (2 340 observaciones; variables: cash-in/transfer-out, etapa del lavado, hora, día). Accuracy ~77 % (NB y RF), ANN 80 %; precisión 0,87, recall 0,72 (RF). Útil para P2 (variables de hora/día y etapa). Falta cuartil (J. of Applied Security Research). No poner 'Sigue' en ronda 5 hasta tener cuartil (la fórmula aprobaría sin él).</t>
+      </text>
+    </comment>
+    <comment ref="L29" authorId="4" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): datos reales de 565 000 transferencias de una caja rural de España, RF supera a redes neuronales y Naive Bayes. Pero es FRAUDE, no lavado ni operaciones inusuales, y reporta 'accuracy 100 %' para legítimas (señal de métrica mal elegida). Ronda 4: dudoso, probablemente Sale. Relevancia baja-media.</t>
       </text>
@@ -381,7 +392,7 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="N29" authorId="2" shapeId="0">
+    <comment ref="N29" authorId="3" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: Sale (ronda 4). Fraude en transferencias (estafas) en una caja rural de España, 565 000 transferencias de 6 semanas, solo 333 fraudes (95 en test). RF: 0 falsos positivos y 91/95 fraudes. No es lavado ni operaciones inusuales; la guía lo excluye. Además no describe variables ni partición temporal, y 0 FP con 95 positivos es poco creíble.</t>
       </text>
@@ -396,18 +407,18 @@
         <t>Implicancias legales</t>
       </text>
     </comment>
-    <comment ref="M37" authorId="3" shapeId="0">
+    <comment ref="M37" authorId="4" shapeId="0">
       <text>
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.
 Corrección: NO es de acceso abierto (licencia solo de minería de texto). Pedirlo por biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M39" authorId="1" shapeId="0">
+    <comment ref="M39" authorId="2" shapeId="0">
       <text>
         <t>Scimago: Expert Systems with Applications, Q1 en 2025. Falta leer el PDF (rondas 4 y 5).</t>
       </text>
     </comment>
-    <comment ref="N39" authorId="1" shapeId="0">
+    <comment ref="N39" authorId="2" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: CUMPLE (Q1). Pese a decir 'fraud', predice eventos SAR (reporte de operación sospechosa de lavado) a partir de alertas SAM de un banco real de Taiwán, con escenarios definidos según la tipología oficial de LA/FT del regulador. Convierte transacciones irregulares de los 15 días hábiles previos en series regulares, autoencoder con self-attention + GNN de relaciones entre clientes + generación de casos (CVAE/WGAN) para el desbalance. Supervisado (etiqueta = decisión del área legal). Compara con XGBoost y redes profundas: AUPRC 27 % vs 0,66-22,15 % (SAR desde alertas) y 22,9 % vs 2,5-22 % (SAR fuera de alertas). Limitación: un solo banco; requiere relaciones entre clientes. Útil para P2 (variables de ventana temporal), P3, P4 y P5 (AUPRC con datos reales y desbalance).</t>
       </text>
@@ -417,12 +428,17 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M43" authorId="1" shapeId="0">
+    <comment ref="N41" authorId="1" shapeId="0">
+      <text>
+        <t>LECTURA COMPLETA: cumple en lo formal pero DÉBIL y de tema dudoso. Sambandam (2025), India. Ontología espacial + reglas SWRL + autoencoder apilado para clasificar transacciones anormales. Datos: dataset financiero SINTÉTICO y dataset de tarjetas de crédito (benchmarks). Accuracy 93 % y 96,23 %. Más cerca de fraude que de lavado. Falta cuartil (Knowledge and Information Systems).</t>
+      </text>
+    </comment>
+    <comment ref="M43" authorId="2" shapeId="0">
       <text>
         <t>Journal of Money Laundering Control 2023: Q2 en Economics, Econometrics and Finance (misc.). Falta leer el PDF.</t>
       </text>
     </comment>
-    <comment ref="N43" authorId="4" shapeId="0">
+    <comment ref="N43" authorId="5" shapeId="0">
       <text>
         <t>LECTURA COMPLETA: cumple en lo formal pero DÉBIL -&gt; RESERVA. JMLC 2023 (Q2). Capitol Technology Univ., EE. UU. Árbol de decisión y otros clasificadores para predecir si una transacción sobre el umbral debe reportarse (SAR). Datos SINTÉTICOS (transacciones públicas 'modificadas' para imitar banca minorista de EE. UU.), un solo escenario AML, balanceo con ROSE. Aporte: identifica atributos relevantes para el SAR (P2). Es de 2023 (límite CE2).</t>
       </text>
@@ -442,7 +458,7 @@
         <t>Es un survey (CE3)</t>
       </text>
     </comment>
-    <comment ref="L52" authorId="2" shapeId="0">
+    <comment ref="L52" authorId="3" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; acceso abierto pero descarga bloqueada): propone un escenario de evaluación realista (banco marca -&gt; autoridad analiza) y muestra que los métodos de punta pierden eficacia; útil para P5. No dice qué datos usa (posible dataset sintético). Ojo cuartil: Royal Society Open Science es multidisciplinaria; Scimago puede no tener categoría de computación/finanzas. Relevancia media.
 LECTURA COMPLETA: cumple en lo formal (aporte + experimentos), pero relevancia BAJA-MEDIA. Dinamarca. Solo datos SINTÉTICOS (IBM-AML) y modelos de grafos (FraudGT, GatedGCN) entre muchos bancos. Hallazgo útil para P5: cuando cada entidad ve solo sus datos, el F1 cae de 0,32/0,71 a 0,12/0,56 y los modelos más simples rinden mejor (0,49/0,85). Perumoney es una sola entidad sin grafo entre cuentas. Recomendación: dejarlo de RESERVA; solo entra si faltan artículos y el cuartil es Q1/Q2.</t>
@@ -458,7 +474,7 @@
         <t>PDF leído. FinCEN Files (SAR filtradas, 1999-2017), Reino Unido. Compara supervisados (RF/XGBoost AUC ~0,97) vs Isolation Forest/One-Class SVM (&lt;0,75): útil para P4. Debilidades: la etiqueta la construyen ellos con su propio score de riesgo (parcialmente circular), test de solo 41 casos, transacciones banco-a-banco. Falta cuartil (IEEE Access). Ronda 4: dudoso.</t>
       </text>
     </comment>
-    <comment ref="M55" authorId="1" shapeId="0">
+    <comment ref="M55" authorId="2" shapeId="0">
       <text>
         <t>IEEE Access 2026: aún no publicado; 2025 = Q1. Artículo de reserva (dudoso en ronda 4).</t>
       </text>
@@ -468,7 +484,7 @@
         <t>Es un review (CE3)</t>
       </text>
     </comment>
-    <comment ref="L81" authorId="2" shapeId="0">
+    <comment ref="L81" authorId="3" shapeId="0">
       <text>
         <t>PRE-EVALUACIÓN (resumen; versión del autor libre pero descarga bloqueada): construcción de grafos dinámicos para GNN en 'financial anomaly detection' sobre datasets de referencia no identificados en el resumen. Requiere grafo de transacciones entre cuentas, que Perumoney no tiene (compra-venta de divisas en ventanilla). Relevancia baja; revisar si los datasets son de cripto (CE4).
 LECTURA COMPLETA (versión aceptada del autor): cumple en lo formal, relevancia BAJA. Malasia/China. Método genérico para construir grafos dinámicos para GNN; prueba con un dataset AML privado (30 M transacciones, origen no declarado), un dataset de crédito alemán y Airbnb. No es cripto (CE4 no aplica). Requiere grafo de transacciones entre cuentas que Perumoney no tiene. Recomendación: Sale en ronda 4.</t>
@@ -1329,7 +1345,11 @@
         </is>
       </c>
       <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
       <c r="O8" s="11" t="n"/>
       <c r="P8" s="8">
         <f>IF(J8="","",IF(K8="Sale","Descartado",IF(L8="Sale","Descartado",IF(OR(M8="Q3",M8="Q4",M8="No aparece"),"Descartado",IF(N8="Sale","Descartado",IF(O8="Sigue","APROBADO","En proceso"))))))</f>
@@ -2659,7 +2679,11 @@
         </is>
       </c>
       <c r="M27" s="11" t="n"/>
-      <c r="N27" s="11" t="n"/>
+      <c r="N27" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="O27" s="11" t="n"/>
       <c r="P27" s="8">
         <f>IF(J27="","",IF(K27="Sale","Descartado",IF(L27="Sale","Descartado",IF(OR(M27="Q3",M27="Q4",M27="No aparece"),"Descartado",IF(N27="Sale","Descartado",IF(O27="Sigue","APROBADO","En proceso"))))))</f>
@@ -3643,7 +3667,11 @@
         </is>
       </c>
       <c r="M41" s="11" t="n"/>
-      <c r="N41" s="11" t="n"/>
+      <c r="N41" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="O41" s="11" t="n"/>
       <c r="P41" s="8">
         <f>IF(J41="","",IF(K41="Sale","Descartado",IF(L41="Sale","Descartado",IF(OR(M41="Q3",M41="Q4",M41="No aparece"),"Descartado",IF(N41="Sale","Descartado",IF(O41="Sigue","APROBADO","En proceso"))))))</f>

</xml_diff>

<commit_message>
Matriz de Joaquín completa: 12 artículos con PDF y cuartil Q1/Q2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Candidatos_Joaquin.xlsx
+++ b/Joaquin/Candidatos_Joaquin.xlsx
@@ -372,9 +372,9 @@
         <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
       </text>
     </comment>
-    <comment ref="M27" authorId="0" shapeId="0">
+    <comment ref="M27" authorId="1" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Journal of Applied Security Research 2024: Q2 en Education, Law, Safety Research y Safety, Risk, Reliability and Quality.</t>
       </text>
     </comment>
     <comment ref="N27" authorId="1" shapeId="0">
@@ -423,9 +423,9 @@
         <t>LECTURA COMPLETA: CUMPLE (Q1). Pese a decir 'fraud', predice eventos SAR (reporte de operación sospechosa de lavado) a partir de alertas SAM de un banco real de Taiwán, con escenarios definidos según la tipología oficial de LA/FT del regulador. Convierte transacciones irregulares de los 15 días hábiles previos en series regulares, autoencoder con self-attention + GNN de relaciones entre clientes + generación de casos (CVAE/WGAN) para el desbalance. Supervisado (etiqueta = decisión del área legal). Compara con XGBoost y redes profundas: AUPRC 27 % vs 0,66-22,15 % (SAR desde alertas) y 22,9 % vs 2,5-22 % (SAR fuera de alertas). Limitación: un solo banco; requiere relaciones entre clientes. Útil para P2 (variables de ventana temporal), P3, P4 y P5 (AUPRC con datos reales y desbalance).</t>
       </text>
     </comment>
-    <comment ref="M41" authorId="0" shapeId="0">
+    <comment ref="M41" authorId="1" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Knowledge and Information Systems 2025: Q2 en Artificial Intelligence (Q1 en Information Systems). Queda de RESERVA: no se registra en la Matriz.</t>
       </text>
     </comment>
     <comment ref="N41" authorId="1" shapeId="0">
@@ -464,9 +464,9 @@
 LECTURA COMPLETA: cumple en lo formal (aporte + experimentos), pero relevancia BAJA-MEDIA. Dinamarca. Solo datos SINTÉTICOS (IBM-AML) y modelos de grafos (FraudGT, GatedGCN) entre muchos bancos. Hallazgo útil para P5: cuando cada entidad ve solo sus datos, el F1 cae de 0,32/0,71 a 0,12/0,56 y los modelos más simples rinden mejor (0,49/0,85). Perumoney es una sola entidad sin grafo entre cuentas. Recomendación: dejarlo de RESERVA; solo entra si faltan artículos y el cuartil es Q1/Q2.</t>
       </text>
     </comment>
-    <comment ref="M52" authorId="0" shapeId="0">
+    <comment ref="M52" authorId="1" shapeId="0">
       <text>
-        <t>PDF no descargado (de pago o bloqueado). Pendiente: cuartil y PDF desde biblioteca UPC.</t>
+        <t>Royal Society Open Science 2025: Q1 en su única categoría (Multidisciplinary). No tiene categoría de computación/finanzas; se usa la única disponible.</t>
       </text>
     </comment>
     <comment ref="L55" authorId="0" shapeId="0">
@@ -2678,13 +2678,21 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M27" s="11" t="n"/>
+      <c r="M27" s="11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="N27" s="11" t="inlineStr">
         <is>
           <t>Sigue</t>
         </is>
       </c>
-      <c r="O27" s="11" t="n"/>
+      <c r="O27" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P27" s="8">
         <f>IF(J27="","",IF(K27="Sale","Descartado",IF(L27="Sale","Descartado",IF(OR(M27="Q3",M27="Q4",M27="No aparece"),"Descartado",IF(N27="Sale","Descartado",IF(O27="Sigue","APROBADO","En proceso"))))))</f>
         <v/>
@@ -3666,7 +3674,11 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M41" s="11" t="n"/>
+      <c r="M41" s="11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
           <t>Sigue</t>
@@ -4436,9 +4448,21 @@
           <t>Sigue</t>
         </is>
       </c>
-      <c r="M52" s="11" t="n"/>
-      <c r="N52" s="11" t="n"/>
-      <c r="O52" s="11" t="n"/>
+      <c r="M52" s="11" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="N52" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
+      <c r="O52" s="11" t="inlineStr">
+        <is>
+          <t>Sigue</t>
+        </is>
+      </c>
       <c r="P52" s="8">
         <f>IF(J52="","",IF(K52="Sale","Descartado",IF(L52="Sale","Descartado",IF(OR(M52="Q3",M52="Q4",M52="No aparece"),"Descartado",IF(N52="Sale","Descartado",IF(O52="Sigue","APROBADO","En proceso"))))))</f>
         <v/>

</xml_diff>